<commit_message>
regenerate the wgcna card now that fry and NES test the same baseline contrast
turquoise, brown and blue stay significant with unchanged direction. green and
yellow flip Up->Down at baseline, which is the mismatch the old weights were
hiding: NES had them Down all along. All five modules now agree.
</commit_message>
<xml_diff>
--- a/04_Figures/F05_WGCNA/c_data/F05_supplementary.xlsx
+++ b/04_Figures/F05_WGCNA/c_data/F05_supplementary.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">fry_camera</t>
   </si>
   <si>
-    <t xml:space="preserve">fry (gate) and camera (reported) per module per contrast.</t>
+    <t xml:space="preserve">fry (reported; subject block via duplicateCorrelation) and camera (sensitivity only: takes no block and assumes inter.gene.cor = 0.01, so its p-values are far smaller and are not the figure's test).</t>
   </si>
   <si>
     <t xml:space="preserve">module_omnibus_F</t>
@@ -48865,28 +48865,28 @@
         <v>55</v>
       </c>
       <c r="D2" t="n">
-        <v>0.19381</v>
+        <v>0.1982</v>
       </c>
       <c r="E2" t="n">
-        <v>0.05008</v>
+        <v>0.05464</v>
       </c>
       <c r="F2" t="n">
-        <v>29.62</v>
+        <v>33.5</v>
       </c>
       <c r="G2" t="n">
-        <v>3.8699</v>
+        <v>3.6273</v>
       </c>
       <c r="H2" t="n">
-        <v>0.000553970978007023</v>
+        <v>0.000942222177605499</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5795</v>
+        <v>0.5311</v>
       </c>
       <c r="J2" t="b">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.00664765173608427</v>
+        <v>0.010851058482229</v>
       </c>
     </row>
     <row r="3">
@@ -48921,7 +48921,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.856655841617893</v>
+        <v>0.852608128569409</v>
       </c>
     </row>
     <row r="4">
@@ -48935,28 +48935,28 @@
         <v>55</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02427</v>
+        <v>-0.01381</v>
       </c>
       <c r="E4" t="n">
-        <v>0.06078</v>
+        <v>0.06738</v>
       </c>
       <c r="F4" t="n">
-        <v>31.16</v>
+        <v>33.98</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3993</v>
+        <v>-0.205</v>
       </c>
       <c r="H4" t="n">
-        <v>0.692430919271719</v>
+        <v>0.83881101457737</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0713</v>
+        <v>-0.0351</v>
       </c>
       <c r="J4" t="b">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.856655841617893</v>
+        <v>0.852608128569409</v>
       </c>
     </row>
     <row r="5">
@@ -49005,28 +49005,28 @@
         <v>55</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.17532</v>
+        <v>-0.1894</v>
       </c>
       <c r="E6" t="n">
-        <v>0.05146</v>
+        <v>0.05584</v>
       </c>
       <c r="F6" t="n">
-        <v>29.1</v>
+        <v>33.19</v>
       </c>
       <c r="G6" t="n">
-        <v>-3.4073</v>
+        <v>-3.3921</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00193731655996856</v>
+        <v>0.00180850974703816</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.534</v>
+        <v>-0.5074</v>
       </c>
       <c r="J6" t="b">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0116238993598114</v>
+        <v>0.010851058482229</v>
       </c>
     </row>
     <row r="7">
@@ -49061,7 +49061,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.827172514709163</v>
+        <v>0.735264457519256</v>
       </c>
     </row>
     <row r="8">
@@ -49075,28 +49075,28 @@
         <v>55</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.15139</v>
+        <v>-0.17503</v>
       </c>
       <c r="E8" t="n">
-        <v>0.05346</v>
+        <v>0.05678</v>
       </c>
       <c r="F8" t="n">
-        <v>27.26</v>
+        <v>31.39</v>
       </c>
       <c r="G8" t="n">
-        <v>-2.8318</v>
+        <v>-3.0827</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00859667985272887</v>
+        <v>0.00425088254196529</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.4768</v>
+        <v>-0.482</v>
       </c>
       <c r="J8" t="b">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0343867194109155</v>
+        <v>0.0170035301678612</v>
       </c>
     </row>
     <row r="9">
@@ -49145,28 +49145,28 @@
         <v>55</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.01745</v>
+        <v>-0.06026</v>
       </c>
       <c r="E10" t="n">
-        <v>0.06021</v>
+        <v>0.06415</v>
       </c>
       <c r="F10" t="n">
-        <v>27.5</v>
+        <v>31.7</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.2899</v>
+        <v>-0.9394</v>
       </c>
       <c r="H10" t="n">
-        <v>0.774094906476404</v>
+        <v>0.354627029799327</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.0552</v>
+        <v>-0.1646</v>
       </c>
       <c r="J10" t="b">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0.856655841617893</v>
+        <v>0.556182647308728</v>
       </c>
     </row>
     <row r="11">
@@ -49215,28 +49215,28 @@
         <v>55</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01099</v>
+        <v>-0.01585</v>
       </c>
       <c r="E12" t="n">
-        <v>0.06034</v>
+        <v>0.06629</v>
       </c>
       <c r="F12" t="n">
-        <v>30.29</v>
+        <v>33.78</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1822</v>
+        <v>-0.2391</v>
       </c>
       <c r="H12" t="n">
-        <v>0.856655841617893</v>
+        <v>0.812463520545173</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0331</v>
+        <v>-0.0411</v>
       </c>
       <c r="J12" t="b">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.856655841617893</v>
+        <v>0.852608128569409</v>
       </c>
     </row>
     <row r="13">
@@ -49271,7 +49271,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0.635637311209974</v>
+        <v>0.556182647308728</v>
       </c>
     </row>
   </sheetData>
@@ -49328,16 +49328,16 @@
         <v>67</v>
       </c>
       <c r="D2" t="n">
-        <v>0.000318973823348515</v>
+        <v>0.000738604547803386</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00159486911674257</v>
+        <v>0.00369302273901693</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000291521919669147</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000169990076679772</v>
       </c>
       <c r="G2" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000145760959834573</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000084995038339886</v>
       </c>
     </row>
     <row r="3">
@@ -49351,16 +49351,16 @@
         <v>68</v>
       </c>
       <c r="D3" t="n">
-        <v>0.00135883566300377</v>
+        <v>0.00156169195971065</v>
       </c>
       <c r="E3" t="n">
-        <v>0.00339708915750944</v>
+        <v>0.00390422989927663</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000000000000000000000000000000107131631638611</v>
+        <v>0.00000000000000000000000000030180547053981</v>
       </c>
       <c r="G3" t="n">
-        <v>0.000000000000000000000000000000267829079096527</v>
+        <v>0.000000000000000000000000000754513676349525</v>
       </c>
     </row>
     <row r="4">
@@ -49374,62 +49374,62 @@
         <v>68</v>
       </c>
       <c r="D4" t="n">
-        <v>0.00606856947564348</v>
+        <v>0.0038405962570915</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0101142824594058</v>
+        <v>0.00640099376181918</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0000000000000000000000170475772703324</v>
+        <v>0.0000000000000000000000101859449949476</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0000000000000000000000284126287838874</v>
+        <v>0.0000000000000000000000169765749915793</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
         <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" t="n">
-        <v>0.745754189298417</v>
+        <v>0.550016524179006</v>
       </c>
       <c r="E5" t="n">
-        <v>0.932192736623021</v>
+        <v>0.687520655223758</v>
       </c>
       <c r="F5" t="n">
-        <v>0.515840575721766</v>
+        <v>0.244753139095252</v>
       </c>
       <c r="G5" t="n">
-        <v>0.644800719652208</v>
+        <v>0.305941423869065</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
         <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D6" t="n">
-        <v>0.937818485550502</v>
+        <v>0.793460916976894</v>
       </c>
       <c r="E6" t="n">
-        <v>0.937818485550502</v>
+        <v>0.793460916976894</v>
       </c>
       <c r="F6" t="n">
-        <v>0.89154598157295</v>
+        <v>0.776916757209867</v>
       </c>
       <c r="G6" t="n">
-        <v>0.89154598157295</v>
+        <v>0.776916757209867</v>
       </c>
     </row>
     <row r="7">

</xml_diff>